<commit_message>
Add dual-mode international calc (full/net weight split)
- guoji: 全重分摊/净重分摊双算法模式，STEP 2 选择算法卡片，后续步骤未选锁定
- 两模式逐人金额数学一致，输出列不同（5列 vs 3列）
- index 入口同步更新

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/演示/拆配排表吧唧.xlsx
+++ b/演示/拆配排表吧唧.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\RenSheet\演示\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7864449E-FE1D-427C-93E1-F7F15B11A66D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F61DBA2-760E-4169-8E83-2D002EB0E8D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3380" yWindow="60" windowWidth="14420" windowHeight="15220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2500" yWindow="70" windowWidth="14420" windowHeight="15220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="12">
   <si>
     <t>吧唧</t>
   </si>
@@ -65,9 +65,6 @@
   </si>
   <si>
     <t>B</t>
-  </si>
-  <si>
-    <t>B</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -76,10 +73,6 @@
   </si>
   <si>
     <t>A</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>特典</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -405,15 +398,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -430,7 +423,7 @@
         <v>5</v>
       </c>
       <c r="F2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G2" t="s">
         <v>6</v>
@@ -438,247 +431,230 @@
       <c r="H2" t="s">
         <v>8</v>
       </c>
-      <c r="I2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H4" t="s">
-        <v>10</v>
-      </c>
-      <c r="I4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>2</v>
       </c>
       <c r="B5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H5" t="s">
-        <v>10</v>
-      </c>
-      <c r="I5" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>3</v>
       </c>
-      <c r="B6" t="s">
-        <v>12</v>
-      </c>
       <c r="C6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H6" t="s">
-        <v>10</v>
-      </c>
-      <c r="I6" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>4</v>
       </c>
-      <c r="B7" t="s">
-        <v>12</v>
-      </c>
       <c r="C7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H7" t="s">
-        <v>10</v>
-      </c>
-      <c r="I7" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>5</v>
       </c>
-      <c r="B8" t="s">
-        <v>12</v>
-      </c>
-      <c r="C8" t="s">
-        <v>12</v>
-      </c>
       <c r="D8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H8" t="s">
-        <v>10</v>
-      </c>
-      <c r="I8" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>6</v>
       </c>
-      <c r="B9" t="s">
-        <v>12</v>
-      </c>
-      <c r="C9" t="s">
-        <v>12</v>
-      </c>
       <c r="D9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G9" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H9" t="s">
-        <v>10</v>
-      </c>
-      <c r="I9" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>7</v>
       </c>
-      <c r="C10" t="s">
-        <v>12</v>
-      </c>
       <c r="D10" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E10" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F10" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G10" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H10" t="s">
-        <v>10</v>
-      </c>
-      <c r="I10" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>8</v>
       </c>
       <c r="D11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G11" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H11" t="s">
-        <v>10</v>
-      </c>
-      <c r="I11" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="D12" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F12" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G12" t="s">
-        <v>10</v>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F13" t="s">
+        <v>11</v>
+      </c>
+      <c r="G13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F14" t="s">
+        <v>11</v>
+      </c>
+      <c r="G14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F15" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F16" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="17" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F17" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>